<commit_message>
docs: sync Firefox upload parity artifacts
</commit_message>
<xml_diff>
--- a/docs/webbrain-mode-tier-tool-chart.xlsx
+++ b/docs/webbrain-mode-tier-tool-chart.xlsx
@@ -1379,11 +1379,11 @@
       <x:c r="C43" s="51" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="D43" s="53" t="str">
-        <x:v>Chrome</x:v>
-      </x:c>
-      <x:c r="E43" s="53" t="str">
-        <x:v>Chrome</x:v>
+      <x:c r="D43" s="49" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E43" s="49" t="str">
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="F43" s="50" t="str">
         <x:v>No</x:v>

</xml_diff>